<commit_message>
Random Walk&ESG-Fx L1 missing runs of RQ2 for small/medium SPLs are completed.
</commit_message>
<xml_diff>
--- a/files/Cases/BankAccountv2/RQ1_BankAccountv2_perRun.xlsx
+++ b/files/Cases/BankAccountv2/RQ1_BankAccountv2_perRun.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10404"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10419"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/dilekozturk/git/esg-with-feature-expressions/files/Cases/BankAccountv2/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{70F27E97-16EE-9B4A-BF5E-12E507593EB6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BC987289-6FEB-6C44-BEF2-A01C9CA8DE7B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="580" windowWidth="25600" windowHeight="15060" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="580" windowWidth="25600" windowHeight="15060" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="EFG_L2" sheetId="1" r:id="rId1"/>
@@ -260,11 +260,16 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -567,8 +572,12 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:W12"/>
+  <dimension ref="A1:W26"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="4" max="4" width="18.6640625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="18.83203125" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
@@ -1421,6 +1430,42 @@
       <c r="W12" t="s">
         <v>25</v>
       </c>
+    </row>
+    <row r="15" spans="1:23" x14ac:dyDescent="0.2">
+      <c r="E15" s="3"/>
+    </row>
+    <row r="16" spans="1:23" x14ac:dyDescent="0.2">
+      <c r="E16" s="4"/>
+    </row>
+    <row r="17" spans="5:5" x14ac:dyDescent="0.2">
+      <c r="E17" s="4"/>
+    </row>
+    <row r="18" spans="5:5" x14ac:dyDescent="0.2">
+      <c r="E18" s="4"/>
+    </row>
+    <row r="19" spans="5:5" x14ac:dyDescent="0.2">
+      <c r="E19" s="4"/>
+    </row>
+    <row r="20" spans="5:5" x14ac:dyDescent="0.2">
+      <c r="E20" s="4"/>
+    </row>
+    <row r="21" spans="5:5" x14ac:dyDescent="0.2">
+      <c r="E21" s="4"/>
+    </row>
+    <row r="22" spans="5:5" x14ac:dyDescent="0.2">
+      <c r="E22" s="4"/>
+    </row>
+    <row r="23" spans="5:5" x14ac:dyDescent="0.2">
+      <c r="E23" s="4"/>
+    </row>
+    <row r="24" spans="5:5" x14ac:dyDescent="0.2">
+      <c r="E24" s="4"/>
+    </row>
+    <row r="25" spans="5:5" x14ac:dyDescent="0.2">
+      <c r="E25" s="4"/>
+    </row>
+    <row r="26" spans="5:5" x14ac:dyDescent="0.2">
+      <c r="E26" s="4"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -3156,7 +3201,10 @@
   <dimension ref="A1:S12"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="5" max="5" width="14.6640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.33203125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="18.6640625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="15.33203125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="26.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:19" x14ac:dyDescent="0.2">
@@ -3876,6 +3924,28 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1:T12"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="6.1640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="8.6640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.33203125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="18.6640625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="14.6640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="16.33203125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="13" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="8.6640625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="21" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="28.6640625" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="21.1640625" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="19" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="22.5" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="23.33203125" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="24" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="19.83203125" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="27.5" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="22.83203125" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="20.33203125" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="22.5" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
@@ -3940,684 +4010,684 @@
       </c>
     </row>
     <row r="2" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="A2">
+      <c r="A2" s="2">
         <v>1</v>
       </c>
-      <c r="B2" t="s">
-        <v>23</v>
-      </c>
-      <c r="C2" t="s">
+      <c r="B2" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="C2" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="D2">
+      <c r="D2" s="2">
         <v>26023.02</v>
       </c>
-      <c r="E2">
+      <c r="E2" s="2">
         <v>100</v>
       </c>
-      <c r="F2">
-        <v>498</v>
-      </c>
-      <c r="G2">
-        <v>0</v>
-      </c>
-      <c r="H2" t="s">
+      <c r="F2" s="2">
+        <v>498</v>
+      </c>
+      <c r="G2" s="2">
+        <v>0</v>
+      </c>
+      <c r="H2" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="I2">
+      <c r="I2" s="2">
         <v>15850</v>
       </c>
-      <c r="J2">
+      <c r="J2" s="2">
         <v>11</v>
       </c>
-      <c r="K2">
-        <v>12660</v>
-      </c>
-      <c r="L2">
-        <v>16395</v>
-      </c>
-      <c r="M2">
+      <c r="K2" s="2">
+        <v>12660</v>
+      </c>
+      <c r="L2" s="2">
+        <v>16395</v>
+      </c>
+      <c r="M2" s="2">
         <v>4407</v>
       </c>
-      <c r="N2">
+      <c r="N2" s="2">
         <v>16506</v>
       </c>
-      <c r="O2">
+      <c r="O2" s="2">
         <v>2486.86</v>
       </c>
-      <c r="P2">
+      <c r="P2" s="2">
         <v>113.49</v>
       </c>
-      <c r="Q2">
+      <c r="Q2" s="2">
         <v>2.7</v>
       </c>
-      <c r="R2">
+      <c r="R2" s="2">
         <v>2705.91</v>
       </c>
-      <c r="S2">
+      <c r="S2" s="2">
         <v>1973.49</v>
       </c>
-      <c r="T2">
+      <c r="T2" s="2">
         <v>2893.26</v>
       </c>
     </row>
     <row r="3" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="A3">
+      <c r="A3" s="2">
         <v>2</v>
       </c>
-      <c r="B3" t="s">
-        <v>23</v>
-      </c>
-      <c r="C3" t="s">
+      <c r="B3" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="C3" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="D3">
+      <c r="D3" s="2">
         <v>28765.37</v>
       </c>
-      <c r="E3">
+      <c r="E3" s="2">
         <v>100</v>
       </c>
-      <c r="F3">
-        <v>498</v>
-      </c>
-      <c r="G3">
-        <v>0</v>
-      </c>
-      <c r="H3" t="s">
+      <c r="F3" s="2">
+        <v>498</v>
+      </c>
+      <c r="G3" s="2">
+        <v>0</v>
+      </c>
+      <c r="H3" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="I3">
+      <c r="I3" s="2">
         <v>17680.400000000001</v>
       </c>
-      <c r="J3">
+      <c r="J3" s="2">
         <v>11</v>
       </c>
-      <c r="K3">
-        <v>12660</v>
-      </c>
-      <c r="L3">
-        <v>16395</v>
-      </c>
-      <c r="M3">
+      <c r="K3" s="2">
+        <v>12660</v>
+      </c>
+      <c r="L3" s="2">
+        <v>16395</v>
+      </c>
+      <c r="M3" s="2">
         <v>4407</v>
       </c>
-      <c r="N3">
+      <c r="N3" s="2">
         <v>16506</v>
       </c>
-      <c r="O3">
+      <c r="O3" s="2">
         <v>2826.3</v>
       </c>
-      <c r="P3">
+      <c r="P3" s="2">
         <v>169.25</v>
       </c>
-      <c r="Q3">
+      <c r="Q3" s="2">
         <v>2.7</v>
       </c>
-      <c r="R3">
+      <c r="R3" s="2">
         <v>2879.89</v>
       </c>
-      <c r="S3">
+      <c r="S3" s="2">
         <v>2389.14</v>
       </c>
-      <c r="T3">
+      <c r="T3" s="2">
         <v>2820.43</v>
       </c>
     </row>
     <row r="4" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="A4">
+      <c r="A4" s="2">
         <v>3</v>
       </c>
-      <c r="B4" t="s">
-        <v>23</v>
-      </c>
-      <c r="C4" t="s">
+      <c r="B4" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="C4" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="D4">
+      <c r="D4" s="2">
         <v>25697.23</v>
       </c>
-      <c r="E4">
+      <c r="E4" s="2">
         <v>100</v>
       </c>
-      <c r="F4">
-        <v>498</v>
-      </c>
-      <c r="G4">
-        <v>0</v>
-      </c>
-      <c r="H4" t="s">
+      <c r="F4" s="2">
+        <v>498</v>
+      </c>
+      <c r="G4" s="2">
+        <v>0</v>
+      </c>
+      <c r="H4" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="I4">
+      <c r="I4" s="2">
         <v>15620.51</v>
       </c>
-      <c r="J4">
+      <c r="J4" s="2">
         <v>11</v>
       </c>
-      <c r="K4">
-        <v>12660</v>
-      </c>
-      <c r="L4">
-        <v>16395</v>
-      </c>
-      <c r="M4">
+      <c r="K4" s="2">
+        <v>12660</v>
+      </c>
+      <c r="L4" s="2">
+        <v>16395</v>
+      </c>
+      <c r="M4" s="2">
         <v>4407</v>
       </c>
-      <c r="N4">
+      <c r="N4" s="2">
         <v>16506</v>
       </c>
-      <c r="O4">
+      <c r="O4" s="2">
         <v>2436.04</v>
       </c>
-      <c r="P4">
+      <c r="P4" s="2">
         <v>111.49</v>
       </c>
-      <c r="Q4">
+      <c r="Q4" s="2">
         <v>2.7</v>
       </c>
-      <c r="R4">
+      <c r="R4" s="2">
         <v>2889.99</v>
       </c>
-      <c r="S4">
+      <c r="S4" s="2">
         <v>1955.12</v>
       </c>
-      <c r="T4">
+      <c r="T4" s="2">
         <v>2684.13</v>
       </c>
     </row>
     <row r="5" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="A5">
+      <c r="A5" s="2">
         <v>4</v>
       </c>
-      <c r="B5" t="s">
-        <v>23</v>
-      </c>
-      <c r="C5" t="s">
+      <c r="B5" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="C5" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="D5">
+      <c r="D5" s="2">
         <v>25537.7</v>
       </c>
-      <c r="E5">
+      <c r="E5" s="2">
         <v>100</v>
       </c>
-      <c r="F5">
-        <v>498</v>
-      </c>
-      <c r="G5">
-        <v>0</v>
-      </c>
-      <c r="H5" t="s">
+      <c r="F5" s="2">
+        <v>498</v>
+      </c>
+      <c r="G5" s="2">
+        <v>0</v>
+      </c>
+      <c r="H5" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="I5">
+      <c r="I5" s="2">
         <v>15379.41</v>
       </c>
-      <c r="J5">
+      <c r="J5" s="2">
         <v>11</v>
       </c>
-      <c r="K5">
-        <v>12660</v>
-      </c>
-      <c r="L5">
-        <v>16395</v>
-      </c>
-      <c r="M5">
+      <c r="K5" s="2">
+        <v>12660</v>
+      </c>
+      <c r="L5" s="2">
+        <v>16395</v>
+      </c>
+      <c r="M5" s="2">
         <v>4407</v>
       </c>
-      <c r="N5">
+      <c r="N5" s="2">
         <v>16506</v>
       </c>
-      <c r="O5">
+      <c r="O5" s="2">
         <v>2482.73</v>
       </c>
-      <c r="P5">
+      <c r="P5" s="2">
         <v>114.72</v>
       </c>
-      <c r="Q5">
+      <c r="Q5" s="2">
         <v>2.7</v>
       </c>
-      <c r="R5">
+      <c r="R5" s="2">
         <v>2667.9</v>
       </c>
-      <c r="S5">
+      <c r="S5" s="2">
         <v>2094.58</v>
       </c>
-      <c r="T5">
+      <c r="T5" s="2">
         <v>2798.3</v>
       </c>
     </row>
     <row r="6" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="A6">
+      <c r="A6" s="2">
         <v>5</v>
       </c>
-      <c r="B6" t="s">
-        <v>23</v>
-      </c>
-      <c r="C6" t="s">
+      <c r="B6" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="C6" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="D6">
+      <c r="D6" s="2">
         <v>27144.84</v>
       </c>
-      <c r="E6">
+      <c r="E6" s="2">
         <v>100</v>
       </c>
-      <c r="F6">
-        <v>498</v>
-      </c>
-      <c r="G6">
-        <v>0</v>
-      </c>
-      <c r="H6" t="s">
+      <c r="F6" s="2">
+        <v>498</v>
+      </c>
+      <c r="G6" s="2">
+        <v>0</v>
+      </c>
+      <c r="H6" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="I6">
+      <c r="I6" s="2">
         <v>16100.82</v>
       </c>
-      <c r="J6">
+      <c r="J6" s="2">
         <v>11</v>
       </c>
-      <c r="K6">
-        <v>12660</v>
-      </c>
-      <c r="L6">
-        <v>16395</v>
-      </c>
-      <c r="M6">
+      <c r="K6" s="2">
+        <v>12660</v>
+      </c>
+      <c r="L6" s="2">
+        <v>16395</v>
+      </c>
+      <c r="M6" s="2">
         <v>4407</v>
       </c>
-      <c r="N6">
+      <c r="N6" s="2">
         <v>16506</v>
       </c>
-      <c r="O6">
+      <c r="O6" s="2">
         <v>2745.05</v>
       </c>
-      <c r="P6">
+      <c r="P6" s="2">
         <v>115.19</v>
       </c>
-      <c r="Q6">
+      <c r="Q6" s="2">
         <v>2.7</v>
       </c>
-      <c r="R6">
+      <c r="R6" s="2">
         <v>3022.19</v>
       </c>
-      <c r="S6">
+      <c r="S6" s="2">
         <v>2188.54</v>
       </c>
-      <c r="T6">
+      <c r="T6" s="2">
         <v>2973.05</v>
       </c>
     </row>
     <row r="7" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="A7">
+      <c r="A7" s="2">
         <v>6</v>
       </c>
-      <c r="B7" t="s">
-        <v>23</v>
-      </c>
-      <c r="C7" t="s">
+      <c r="B7" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="C7" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="D7">
+      <c r="D7" s="2">
         <v>27914.52</v>
       </c>
-      <c r="E7">
+      <c r="E7" s="2">
         <v>100</v>
       </c>
-      <c r="F7">
-        <v>498</v>
-      </c>
-      <c r="G7">
-        <v>0</v>
-      </c>
-      <c r="H7" t="s">
+      <c r="F7" s="2">
+        <v>498</v>
+      </c>
+      <c r="G7" s="2">
+        <v>0</v>
+      </c>
+      <c r="H7" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="I7">
+      <c r="I7" s="2">
         <v>17155.650000000001</v>
       </c>
-      <c r="J7">
+      <c r="J7" s="2">
         <v>11</v>
       </c>
-      <c r="K7">
-        <v>12660</v>
-      </c>
-      <c r="L7">
-        <v>16395</v>
-      </c>
-      <c r="M7">
+      <c r="K7" s="2">
+        <v>12660</v>
+      </c>
+      <c r="L7" s="2">
+        <v>16395</v>
+      </c>
+      <c r="M7" s="2">
         <v>4407</v>
       </c>
-      <c r="N7">
+      <c r="N7" s="2">
         <v>16506</v>
       </c>
-      <c r="O7">
+      <c r="O7" s="2">
         <v>2707.4</v>
       </c>
-      <c r="P7">
+      <c r="P7" s="2">
         <v>150.27000000000001</v>
       </c>
-      <c r="Q7">
+      <c r="Q7" s="2">
         <v>2.7</v>
       </c>
-      <c r="R7">
+      <c r="R7" s="2">
         <v>2873.1</v>
       </c>
-      <c r="S7">
+      <c r="S7" s="2">
         <v>2248.5700000000002</v>
       </c>
-      <c r="T7">
+      <c r="T7" s="2">
         <v>2779.56</v>
       </c>
     </row>
     <row r="8" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="A8">
+      <c r="A8" s="2">
         <v>7</v>
       </c>
-      <c r="B8" t="s">
-        <v>23</v>
-      </c>
-      <c r="C8" t="s">
+      <c r="B8" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="C8" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="D8">
+      <c r="D8" s="2">
         <v>25520.080000000002</v>
       </c>
-      <c r="E8">
+      <c r="E8" s="2">
         <v>100</v>
       </c>
-      <c r="F8">
-        <v>498</v>
-      </c>
-      <c r="G8">
-        <v>0</v>
-      </c>
-      <c r="H8" t="s">
+      <c r="F8" s="2">
+        <v>498</v>
+      </c>
+      <c r="G8" s="2">
+        <v>0</v>
+      </c>
+      <c r="H8" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="I8">
+      <c r="I8" s="2">
         <v>15366.5</v>
       </c>
-      <c r="J8">
+      <c r="J8" s="2">
         <v>11</v>
       </c>
-      <c r="K8">
-        <v>12660</v>
-      </c>
-      <c r="L8">
-        <v>16395</v>
-      </c>
-      <c r="M8">
+      <c r="K8" s="2">
+        <v>12660</v>
+      </c>
+      <c r="L8" s="2">
+        <v>16395</v>
+      </c>
+      <c r="M8" s="2">
         <v>4407</v>
       </c>
-      <c r="N8">
+      <c r="N8" s="2">
         <v>16506</v>
       </c>
-      <c r="O8">
+      <c r="O8" s="2">
         <v>2493.7399999999998</v>
       </c>
-      <c r="P8">
+      <c r="P8" s="2">
         <v>146.43</v>
       </c>
-      <c r="Q8">
+      <c r="Q8" s="2">
         <v>2.7</v>
       </c>
-      <c r="R8">
+      <c r="R8" s="2">
         <v>2682.86</v>
       </c>
-      <c r="S8">
+      <c r="S8" s="2">
         <v>2117.71</v>
       </c>
-      <c r="T8">
+      <c r="T8" s="2">
         <v>2712.74</v>
       </c>
     </row>
     <row r="9" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="A9">
+      <c r="A9" s="2">
         <v>8</v>
       </c>
-      <c r="B9" t="s">
-        <v>23</v>
-      </c>
-      <c r="C9" t="s">
+      <c r="B9" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="C9" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="D9">
+      <c r="D9" s="2">
         <v>26874.93</v>
       </c>
-      <c r="E9">
+      <c r="E9" s="2">
         <v>100</v>
       </c>
-      <c r="F9">
-        <v>498</v>
-      </c>
-      <c r="G9">
-        <v>0</v>
-      </c>
-      <c r="H9" t="s">
+      <c r="F9" s="2">
+        <v>498</v>
+      </c>
+      <c r="G9" s="2">
+        <v>0</v>
+      </c>
+      <c r="H9" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="I9">
+      <c r="I9" s="2">
         <v>16418.740000000002</v>
       </c>
-      <c r="J9">
+      <c r="J9" s="2">
         <v>11</v>
       </c>
-      <c r="K9">
-        <v>12660</v>
-      </c>
-      <c r="L9">
-        <v>16395</v>
-      </c>
-      <c r="M9">
+      <c r="K9" s="2">
+        <v>12660</v>
+      </c>
+      <c r="L9" s="2">
+        <v>16395</v>
+      </c>
+      <c r="M9" s="2">
         <v>4407</v>
       </c>
-      <c r="N9">
+      <c r="N9" s="2">
         <v>16506</v>
       </c>
-      <c r="O9">
+      <c r="O9" s="2">
         <v>2563.29</v>
       </c>
-      <c r="P9">
+      <c r="P9" s="2">
         <v>128.77000000000001</v>
       </c>
-      <c r="Q9">
+      <c r="Q9" s="2">
         <v>2.7</v>
       </c>
-      <c r="R9">
+      <c r="R9" s="2">
         <v>2938.88</v>
       </c>
-      <c r="S9">
+      <c r="S9" s="2">
         <v>2076.4499999999998</v>
       </c>
-      <c r="T9">
+      <c r="T9" s="2">
         <v>2748.83</v>
       </c>
     </row>
     <row r="10" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="A10">
+      <c r="A10" s="2">
         <v>9</v>
       </c>
-      <c r="B10" t="s">
-        <v>23</v>
-      </c>
-      <c r="C10" t="s">
+      <c r="B10" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="C10" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="D10">
+      <c r="D10" s="2">
         <v>25496.67</v>
       </c>
-      <c r="E10">
+      <c r="E10" s="2">
         <v>100</v>
       </c>
-      <c r="F10">
-        <v>498</v>
-      </c>
-      <c r="G10">
-        <v>0</v>
-      </c>
-      <c r="H10" t="s">
+      <c r="F10" s="2">
+        <v>498</v>
+      </c>
+      <c r="G10" s="2">
+        <v>0</v>
+      </c>
+      <c r="H10" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="I10">
+      <c r="I10" s="2">
         <v>15673.24</v>
       </c>
-      <c r="J10">
+      <c r="J10" s="2">
         <v>11</v>
       </c>
-      <c r="K10">
-        <v>12660</v>
-      </c>
-      <c r="L10">
-        <v>16395</v>
-      </c>
-      <c r="M10">
+      <c r="K10" s="2">
+        <v>12660</v>
+      </c>
+      <c r="L10" s="2">
+        <v>16395</v>
+      </c>
+      <c r="M10" s="2">
         <v>4407</v>
       </c>
-      <c r="N10">
+      <c r="N10" s="2">
         <v>16506</v>
       </c>
-      <c r="O10">
+      <c r="O10" s="2">
         <v>2256.14</v>
       </c>
-      <c r="P10">
+      <c r="P10" s="2">
         <v>118.08</v>
       </c>
-      <c r="Q10">
+      <c r="Q10" s="2">
         <v>2.7</v>
       </c>
-      <c r="R10">
+      <c r="R10" s="2">
         <v>2716.59</v>
       </c>
-      <c r="S10">
+      <c r="S10" s="2">
         <v>2015.55</v>
       </c>
-      <c r="T10">
+      <c r="T10" s="2">
         <v>2717.05</v>
       </c>
     </row>
     <row r="11" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="A11">
+      <c r="A11" s="2">
         <v>10</v>
       </c>
-      <c r="B11" t="s">
-        <v>23</v>
-      </c>
-      <c r="C11" t="s">
+      <c r="B11" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="C11" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="D11">
+      <c r="D11" s="2">
         <v>27189.32</v>
       </c>
-      <c r="E11">
+      <c r="E11" s="2">
         <v>100</v>
       </c>
-      <c r="F11">
-        <v>498</v>
-      </c>
-      <c r="G11">
-        <v>0</v>
-      </c>
-      <c r="H11" t="s">
+      <c r="F11" s="2">
+        <v>498</v>
+      </c>
+      <c r="G11" s="2">
+        <v>0</v>
+      </c>
+      <c r="H11" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="I11">
+      <c r="I11" s="2">
         <v>16292.65</v>
       </c>
-      <c r="J11">
+      <c r="J11" s="2">
         <v>11</v>
       </c>
-      <c r="K11">
-        <v>12660</v>
-      </c>
-      <c r="L11">
-        <v>16395</v>
-      </c>
-      <c r="M11">
+      <c r="K11" s="2">
+        <v>12660</v>
+      </c>
+      <c r="L11" s="2">
+        <v>16395</v>
+      </c>
+      <c r="M11" s="2">
         <v>4407</v>
       </c>
-      <c r="N11">
+      <c r="N11" s="2">
         <v>16506</v>
       </c>
-      <c r="O11">
+      <c r="O11" s="2">
         <v>2737.57</v>
       </c>
-      <c r="P11">
+      <c r="P11" s="2">
         <v>150.16999999999999</v>
       </c>
-      <c r="Q11">
+      <c r="Q11" s="2">
         <v>2.7</v>
       </c>
-      <c r="R11">
+      <c r="R11" s="2">
         <v>2940.9</v>
       </c>
-      <c r="S11">
+      <c r="S11" s="2">
         <v>2274.64</v>
       </c>
-      <c r="T11">
+      <c r="T11" s="2">
         <v>2793.43</v>
       </c>
     </row>
     <row r="12" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="A12">
+      <c r="A12" s="2">
         <v>11</v>
       </c>
-      <c r="B12" t="s">
-        <v>23</v>
-      </c>
-      <c r="C12" t="s">
+      <c r="B12" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="C12" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="D12">
+      <c r="D12" s="2">
         <v>26267.360000000001</v>
       </c>
-      <c r="E12">
+      <c r="E12" s="2">
         <v>100</v>
       </c>
-      <c r="F12">
-        <v>498</v>
-      </c>
-      <c r="G12">
-        <v>0</v>
-      </c>
-      <c r="H12" t="s">
+      <c r="F12" s="2">
+        <v>498</v>
+      </c>
+      <c r="G12" s="2">
+        <v>0</v>
+      </c>
+      <c r="H12" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="I12">
+      <c r="I12" s="2">
         <v>15568.81</v>
       </c>
-      <c r="J12">
+      <c r="J12" s="2">
         <v>11</v>
       </c>
-      <c r="K12">
-        <v>12660</v>
-      </c>
-      <c r="L12">
-        <v>16395</v>
-      </c>
-      <c r="M12">
+      <c r="K12" s="2">
+        <v>12660</v>
+      </c>
+      <c r="L12" s="2">
+        <v>16395</v>
+      </c>
+      <c r="M12" s="2">
         <v>4407</v>
       </c>
-      <c r="N12">
+      <c r="N12" s="2">
         <v>16506</v>
       </c>
-      <c r="O12">
+      <c r="O12" s="2">
         <v>2605.85</v>
       </c>
-      <c r="P12">
+      <c r="P12" s="2">
         <v>150.35</v>
       </c>
-      <c r="Q12">
+      <c r="Q12" s="2">
         <v>2.7</v>
       </c>
-      <c r="R12">
+      <c r="R12" s="2">
         <v>2800.29</v>
       </c>
-      <c r="S12">
+      <c r="S12" s="2">
         <v>2207.71</v>
       </c>
-      <c r="T12">
+      <c r="T12" s="2">
         <v>2934.48</v>
       </c>
     </row>

</xml_diff>